<commit_message>
Use generic column headers in MetaData template
The "Create MetaData.xlsx" template now labels the Names-sheet header row
"column 1"..."column 12" instead of "blank/sample 1.../standard", matching
the updated Example/MetaData.xlsx. The header describes the 12 physical
plate columns, while the data rows still pre-fill the suggested default
layout (blank, samples, standard).

Also fix header-row detection in parseMetadata(): it previously required
B1 === 'blank', which the new "column 1" header would fail, causing the
header to be misread as plate data. Detection now keys only on
A1 === 'Plate', which stays backward-compatible with old templates.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Example/MetaData.xlsx
+++ b/Example/MetaData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kasimirreich/Documents/Nussenzweig Lab/Data/ELISA/260528_Linvivo_d85_a101074+yu2gp140/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kasimirreich/Documents/Claude Code/ELISA-Workflow-App/Example/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BC07A93-279B-7244-B96A-91543550A46C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{578C5687-28B7-8F44-94DC-A79A1583EDD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="25">
   <si>
     <t>Plate</t>
   </si>
@@ -29,36 +29,6 @@
     <t>blank</t>
   </si>
   <si>
-    <t>sample 1</t>
-  </si>
-  <si>
-    <t>sample 2</t>
-  </si>
-  <si>
-    <t>sample 3</t>
-  </si>
-  <si>
-    <t>sample 4</t>
-  </si>
-  <si>
-    <t>sample 5</t>
-  </si>
-  <si>
-    <t>sample 6</t>
-  </si>
-  <si>
-    <t>sample 7</t>
-  </si>
-  <si>
-    <t>sample 8</t>
-  </si>
-  <si>
-    <t>sample 9</t>
-  </si>
-  <si>
-    <t>sample 10</t>
-  </si>
-  <si>
     <t>standard</t>
   </si>
   <si>
@@ -90,6 +60,42 @@
   </si>
   <si>
     <t>plate 6 - d85 yu2gp142</t>
+  </si>
+  <si>
+    <t>column 1</t>
+  </si>
+  <si>
+    <t>column 2</t>
+  </si>
+  <si>
+    <t>column 3</t>
+  </si>
+  <si>
+    <t>column 4</t>
+  </si>
+  <si>
+    <t>column 5</t>
+  </si>
+  <si>
+    <t>column 6</t>
+  </si>
+  <si>
+    <t>column 7</t>
+  </si>
+  <si>
+    <t>column 8</t>
+  </si>
+  <si>
+    <t>column 9</t>
+  </si>
+  <si>
+    <t>column 10</t>
+  </si>
+  <si>
+    <t>column 11</t>
+  </si>
+  <si>
+    <t>column 12</t>
   </si>
 </sst>
 </file>
@@ -518,45 +524,45 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
@@ -592,12 +598,12 @@
         <v>1</v>
       </c>
       <c r="M2" s="7" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
         <v>1</v>
@@ -633,12 +639,12 @@
         <v>1</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
         <v>1</v>
@@ -674,12 +680,12 @@
         <v>1</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
         <v>1</v>
@@ -715,12 +721,12 @@
         <v>1</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
         <v>1</v>
@@ -756,12 +762,12 @@
         <v>1</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
         <v>1</v>
@@ -797,7 +803,7 @@
         <v>1</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -817,7 +823,7 @@
   <sheetData>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="B2">
         <v>1000</v>
@@ -825,7 +831,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="B3">
         <v>5</v>
@@ -833,7 +839,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="B6">
         <v>50</v>
@@ -841,7 +847,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B7">
         <v>4</v>

</xml_diff>